<commit_message>
BOM items added and more formatting to the ReadMe.
</commit_message>
<xml_diff>
--- a/ReadMe Assets/Dr-Infrared-Heater-Remote-Thermostat BOM.xlsx
+++ b/ReadMe Assets/Dr-Infrared-Heater-Remote-Thermostat BOM.xlsx
@@ -5,10 +5,10 @@
   <workbookPr/>
   <mc:AlternateContent xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006">
     <mc:Choice Requires="x15">
-      <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="C:\Users\talyn\OneDrive\Desktop\Personel Projects\Shop Heater\Public Repo\Dr-Infrared-Heater-Remote-Thermostat\ReadMe Assets\"/>
+      <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="https://d.docs.live.net/d02527ba799f7e57/Desktop/Personel Projects/Shop Heater/Public Repo/Dr-Infrared-Heater-Remote-Thermostat/ReadMe Assets/"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{C3E0A6F9-8DAD-4268-B801-F770A0C7E470}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="105" documentId="13_ncr:1_{C3E0A6F9-8DAD-4268-B801-F770A0C7E470}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{D2E7A27F-CA4A-417F-81CB-854403E51689}"/>
   <bookViews>
     <workbookView xWindow="-28920" yWindow="-90" windowWidth="29040" windowHeight="15720" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
   </bookViews>
@@ -60,7 +60,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="9" uniqueCount="9">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="44" uniqueCount="36">
   <si>
     <t>Description</t>
   </si>
@@ -87,6 +87,87 @@
   </si>
   <si>
     <t>Dr Infrared Heater DR-966</t>
+  </si>
+  <si>
+    <t xml:space="preserve">Grand Total: </t>
+  </si>
+  <si>
+    <t>Digikey</t>
+  </si>
+  <si>
+    <t>Raspberry Pi Zero 2W</t>
+  </si>
+  <si>
+    <t>120-240vac to 5vdc power supply</t>
+  </si>
+  <si>
+    <t xml:space="preserve">	2648-SC0721-ND</t>
+  </si>
+  <si>
+    <t>1866-4133-ND</t>
+  </si>
+  <si>
+    <t>1528-1698-ND</t>
+  </si>
+  <si>
+    <t>Raspberry Pi Heat Sink</t>
+  </si>
+  <si>
+    <t>Raspberry Pi Zero Proto Bonnet Board</t>
+  </si>
+  <si>
+    <t>1528-2041-ND</t>
+  </si>
+  <si>
+    <t>1528-1592-ND</t>
+  </si>
+  <si>
+    <t>Waterproof 1-Wire DS18B20 Digital temperature sensor</t>
+  </si>
+  <si>
+    <t>Dual Channel 5vdc control 240vac 30 Amp Relay Board</t>
+  </si>
+  <si>
+    <t>Amazon</t>
+  </si>
+  <si>
+    <t>B07DSXWPC1</t>
+  </si>
+  <si>
+    <t>McMaster-Carr</t>
+  </si>
+  <si>
+    <t>92005A116</t>
+  </si>
+  <si>
+    <t>Power Supply Phillips Screw</t>
+  </si>
+  <si>
+    <t>Raspberry Pi and Relay Board Phillips Screw</t>
+  </si>
+  <si>
+    <t>92005A052</t>
+  </si>
+  <si>
+    <t>Wago Wire Connector</t>
+  </si>
+  <si>
+    <t>2946-221-613-ND</t>
+  </si>
+  <si>
+    <t>Two Position Terminal Block</t>
+  </si>
+  <si>
+    <t>Three Position Terminal Block</t>
+  </si>
+  <si>
+    <t>277-1273-ND</t>
+  </si>
+  <si>
+    <t>277-1274-ND</t>
+  </si>
+  <si>
+    <t>16 gauge wire and proabbly 20 gauge wire</t>
   </si>
 </sst>
 </file>
@@ -97,7 +178,7 @@
     <numFmt numFmtId="44" formatCode="_(&quot;$&quot;* #,##0.00_);_(&quot;$&quot;* \(#,##0.00\);_(&quot;$&quot;* &quot;-&quot;??_);_(@_)"/>
     <numFmt numFmtId="164" formatCode="&quot;$&quot;#,##0.00"/>
   </numFmts>
-  <fonts count="5" x14ac:knownFonts="1">
+  <fonts count="6" x14ac:knownFonts="1">
     <font>
       <sz val="11"/>
       <color theme="1"/>
@@ -134,8 +215,16 @@
       <family val="2"/>
       <scheme val="minor"/>
     </font>
+    <font>
+      <b/>
+      <sz val="11"/>
+      <color theme="1"/>
+      <name val="Calibri"/>
+      <family val="2"/>
+      <scheme val="minor"/>
+    </font>
   </fonts>
-  <fills count="3">
+  <fills count="4">
     <fill>
       <patternFill patternType="none"/>
     </fill>
@@ -145,6 +234,12 @@
     <fill>
       <patternFill patternType="solid">
         <fgColor theme="0" tint="-0.249977111117893"/>
+        <bgColor indexed="64"/>
+      </patternFill>
+    </fill>
+    <fill>
+      <patternFill patternType="solid">
+        <fgColor theme="5" tint="0.59999389629810485"/>
         <bgColor indexed="64"/>
       </patternFill>
     </fill>
@@ -178,7 +273,7 @@
     <xf numFmtId="44" fontId="1" fillId="0" borderId="0" applyFont="0" applyFill="0" applyBorder="0" applyAlignment="0" applyProtection="0"/>
     <xf numFmtId="0" fontId="3" fillId="0" borderId="0" applyNumberFormat="0" applyFill="0" applyBorder="0" applyAlignment="0" applyProtection="0"/>
   </cellStyleXfs>
-  <cellXfs count="6">
+  <cellXfs count="11">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0"/>
     <xf numFmtId="0" fontId="0" fillId="0" borderId="1" xfId="0" applyBorder="1"/>
     <xf numFmtId="0" fontId="0" fillId="0" borderId="1" xfId="0" applyBorder="1" applyAlignment="1">
@@ -191,6 +286,21 @@
       <alignment horizontal="center" vertical="center"/>
     </xf>
     <xf numFmtId="0" fontId="4" fillId="2" borderId="1" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="5" fillId="3" borderId="1" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="right"/>
+    </xf>
+    <xf numFmtId="0" fontId="0" fillId="3" borderId="1" xfId="0" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="right"/>
+    </xf>
+    <xf numFmtId="164" fontId="5" fillId="0" borderId="1" xfId="0" applyNumberFormat="1" applyFont="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="0" fillId="0" borderId="1" xfId="0" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="3" fillId="0" borderId="0" xfId="2" applyAlignment="1">
       <alignment horizontal="center" vertical="center"/>
     </xf>
   </cellXfs>
@@ -475,7 +585,7 @@
 
 <file path=xl/worksheets/sheet1.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:xdr="http://schemas.openxmlformats.org/drawingml/2006/spreadsheetDrawing" xmlns:x14="http://schemas.microsoft.com/office/spreadsheetml/2009/9/main" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{00000000-0001-0000-0000-000000000000}">
-  <dimension ref="A1:F18"/>
+  <dimension ref="A1:F19"/>
   <sheetFormatPr defaultRowHeight="14.5" x14ac:dyDescent="0.35"/>
   <cols>
     <col min="1" max="1" width="60.6328125" customWidth="1"/>
@@ -525,128 +635,240 @@
       </c>
     </row>
     <row r="3" spans="1:6" x14ac:dyDescent="0.35">
-      <c r="A3" s="1"/>
-      <c r="B3" s="2"/>
-      <c r="C3" s="2"/>
-      <c r="D3" s="2"/>
-      <c r="E3" s="3"/>
+      <c r="A3" s="1" t="s">
+        <v>11</v>
+      </c>
+      <c r="B3" s="9" t="s">
+        <v>13</v>
+      </c>
+      <c r="C3" s="4" t="s">
+        <v>10</v>
+      </c>
+      <c r="D3" s="2">
+        <v>1</v>
+      </c>
+      <c r="E3" s="3">
+        <v>18</v>
+      </c>
       <c r="F3" s="3">
         <f t="shared" ref="F3:F18" si="0">D3*E3</f>
-        <v>0</v>
+        <v>18</v>
       </c>
     </row>
     <row r="4" spans="1:6" x14ac:dyDescent="0.35">
-      <c r="A4" s="1"/>
-      <c r="B4" s="2"/>
-      <c r="C4" s="2"/>
-      <c r="D4" s="2"/>
-      <c r="E4" s="3"/>
+      <c r="A4" s="1" t="s">
+        <v>16</v>
+      </c>
+      <c r="B4" s="2" t="s">
+        <v>15</v>
+      </c>
+      <c r="C4" s="4" t="s">
+        <v>10</v>
+      </c>
+      <c r="D4" s="2">
+        <v>1</v>
+      </c>
+      <c r="E4" s="3">
+        <v>0.95</v>
+      </c>
       <c r="F4" s="3">
         <f t="shared" si="0"/>
-        <v>0</v>
+        <v>0.95</v>
       </c>
     </row>
     <row r="5" spans="1:6" x14ac:dyDescent="0.35">
-      <c r="A5" s="1"/>
-      <c r="B5" s="2"/>
-      <c r="C5" s="2"/>
-      <c r="D5" s="2"/>
-      <c r="E5" s="3"/>
+      <c r="A5" s="1" t="s">
+        <v>17</v>
+      </c>
+      <c r="B5" s="2" t="s">
+        <v>18</v>
+      </c>
+      <c r="C5" s="4" t="s">
+        <v>10</v>
+      </c>
+      <c r="D5" s="2">
+        <v>1</v>
+      </c>
+      <c r="E5" s="3">
+        <v>4.5</v>
+      </c>
       <c r="F5" s="3">
         <f t="shared" si="0"/>
-        <v>0</v>
+        <v>4.5</v>
       </c>
     </row>
     <row r="6" spans="1:6" x14ac:dyDescent="0.35">
-      <c r="A6" s="1"/>
-      <c r="B6" s="2"/>
-      <c r="C6" s="2"/>
-      <c r="D6" s="2"/>
-      <c r="E6" s="3"/>
+      <c r="A6" s="1" t="s">
+        <v>20</v>
+      </c>
+      <c r="B6" s="2" t="s">
+        <v>19</v>
+      </c>
+      <c r="C6" s="4" t="s">
+        <v>10</v>
+      </c>
+      <c r="D6" s="2">
+        <v>1</v>
+      </c>
+      <c r="E6" s="3">
+        <v>9.9499999999999993</v>
+      </c>
       <c r="F6" s="3">
         <f t="shared" si="0"/>
-        <v>0</v>
+        <v>9.9499999999999993</v>
       </c>
     </row>
     <row r="7" spans="1:6" x14ac:dyDescent="0.35">
-      <c r="A7" s="1"/>
-      <c r="B7" s="2"/>
-      <c r="C7" s="2"/>
-      <c r="D7" s="2"/>
-      <c r="E7" s="3"/>
+      <c r="A7" s="1" t="s">
+        <v>31</v>
+      </c>
+      <c r="B7" s="2" t="s">
+        <v>33</v>
+      </c>
+      <c r="C7" s="10" t="s">
+        <v>10</v>
+      </c>
+      <c r="D7" s="2">
+        <v>2</v>
+      </c>
+      <c r="E7" s="3">
+        <v>1.93</v>
+      </c>
       <c r="F7" s="3">
         <f t="shared" si="0"/>
-        <v>0</v>
+        <v>3.86</v>
       </c>
     </row>
     <row r="8" spans="1:6" x14ac:dyDescent="0.35">
-      <c r="A8" s="1"/>
-      <c r="B8" s="2"/>
-      <c r="C8" s="2"/>
-      <c r="D8" s="2"/>
-      <c r="E8" s="3"/>
+      <c r="A8" s="1" t="s">
+        <v>32</v>
+      </c>
+      <c r="B8" s="2" t="s">
+        <v>34</v>
+      </c>
+      <c r="C8" s="4" t="s">
+        <v>10</v>
+      </c>
+      <c r="D8" s="2">
+        <v>2</v>
+      </c>
+      <c r="E8" s="3">
+        <v>2.77</v>
+      </c>
       <c r="F8" s="3">
         <f t="shared" si="0"/>
-        <v>0</v>
+        <v>5.54</v>
       </c>
     </row>
     <row r="9" spans="1:6" x14ac:dyDescent="0.35">
-      <c r="A9" s="1"/>
-      <c r="B9" s="2"/>
-      <c r="C9" s="2"/>
-      <c r="D9" s="2"/>
-      <c r="E9" s="3"/>
+      <c r="A9" s="1" t="s">
+        <v>29</v>
+      </c>
+      <c r="B9" s="2" t="s">
+        <v>30</v>
+      </c>
+      <c r="C9" s="4" t="s">
+        <v>10</v>
+      </c>
+      <c r="D9" s="2">
+        <v>3</v>
+      </c>
+      <c r="E9" s="3">
+        <v>1.22</v>
+      </c>
       <c r="F9" s="3">
         <f t="shared" si="0"/>
-        <v>0</v>
+        <v>3.66</v>
       </c>
     </row>
     <row r="10" spans="1:6" x14ac:dyDescent="0.35">
-      <c r="A10" s="1"/>
-      <c r="B10" s="2"/>
-      <c r="C10" s="2"/>
-      <c r="D10" s="2"/>
-      <c r="E10" s="3"/>
+      <c r="A10" s="1" t="s">
+        <v>12</v>
+      </c>
+      <c r="B10" s="2" t="s">
+        <v>14</v>
+      </c>
+      <c r="C10" s="4" t="s">
+        <v>10</v>
+      </c>
+      <c r="D10" s="2">
+        <v>1</v>
+      </c>
+      <c r="E10" s="3">
+        <v>8.6</v>
+      </c>
       <c r="F10" s="3">
         <f t="shared" si="0"/>
-        <v>0</v>
+        <v>8.6</v>
       </c>
     </row>
     <row r="11" spans="1:6" x14ac:dyDescent="0.35">
-      <c r="A11" s="1"/>
-      <c r="B11" s="2"/>
-      <c r="C11" s="2"/>
-      <c r="D11" s="2"/>
-      <c r="E11" s="3"/>
+      <c r="A11" s="1" t="s">
+        <v>21</v>
+      </c>
+      <c r="B11" s="2" t="s">
+        <v>23</v>
+      </c>
+      <c r="C11" s="4" t="s">
+        <v>22</v>
+      </c>
+      <c r="D11" s="2">
+        <v>1</v>
+      </c>
+      <c r="E11" s="3">
+        <v>10.99</v>
+      </c>
       <c r="F11" s="3">
         <f t="shared" si="0"/>
-        <v>0</v>
+        <v>10.99</v>
       </c>
     </row>
     <row r="12" spans="1:6" x14ac:dyDescent="0.35">
-      <c r="A12" s="1"/>
-      <c r="B12" s="2"/>
-      <c r="C12" s="2"/>
-      <c r="D12" s="2"/>
-      <c r="E12" s="3"/>
+      <c r="A12" s="1" t="s">
+        <v>26</v>
+      </c>
+      <c r="B12" s="2" t="s">
+        <v>25</v>
+      </c>
+      <c r="C12" s="4" t="s">
+        <v>24</v>
+      </c>
+      <c r="D12" s="2">
+        <v>1</v>
+      </c>
+      <c r="E12" s="3">
+        <v>4.4800000000000004</v>
+      </c>
       <c r="F12" s="3">
         <f t="shared" si="0"/>
-        <v>0</v>
+        <v>4.4800000000000004</v>
       </c>
     </row>
     <row r="13" spans="1:6" x14ac:dyDescent="0.35">
-      <c r="A13" s="1"/>
-      <c r="B13" s="2"/>
-      <c r="C13" s="2"/>
-      <c r="D13" s="2"/>
-      <c r="E13" s="3"/>
+      <c r="A13" s="1" t="s">
+        <v>27</v>
+      </c>
+      <c r="B13" s="2" t="s">
+        <v>28</v>
+      </c>
+      <c r="C13" s="4" t="s">
+        <v>24</v>
+      </c>
+      <c r="D13" s="2">
+        <v>1</v>
+      </c>
+      <c r="E13" s="3">
+        <v>6.87</v>
+      </c>
       <c r="F13" s="3">
         <f t="shared" si="0"/>
-        <v>0</v>
+        <v>6.87</v>
       </c>
     </row>
     <row r="14" spans="1:6" x14ac:dyDescent="0.35">
-      <c r="A14" s="1"/>
+      <c r="A14" s="1" t="s">
+        <v>35</v>
+      </c>
       <c r="B14" s="2"/>
       <c r="C14" s="2"/>
       <c r="D14" s="2"/>
@@ -700,11 +922,38 @@
         <v>0</v>
       </c>
     </row>
+    <row r="19" spans="1:6" x14ac:dyDescent="0.35">
+      <c r="A19" s="6" t="s">
+        <v>9</v>
+      </c>
+      <c r="B19" s="7"/>
+      <c r="C19" s="7"/>
+      <c r="D19" s="7"/>
+      <c r="E19" s="7"/>
+      <c r="F19" s="8">
+        <f>SUM(F2:F18)</f>
+        <v>277.39999999999998</v>
+      </c>
+    </row>
   </sheetData>
+  <mergeCells count="1">
+    <mergeCell ref="A19:E19"/>
+  </mergeCells>
   <hyperlinks>
     <hyperlink ref="C2" r:id="rId1" xr:uid="{7E1BCDF3-976F-4AEC-B6D9-914AB11C8929}"/>
+    <hyperlink ref="C3" r:id="rId2" xr:uid="{E9D06958-5AD5-46DF-B69C-3902CC72E8E2}"/>
+    <hyperlink ref="C10" r:id="rId3" xr:uid="{D022BB45-F54B-4EE7-A5EF-F34DA750CE30}"/>
+    <hyperlink ref="C4" r:id="rId4" xr:uid="{DC272C52-B2F4-42A2-A5F6-AD123CB15E40}"/>
+    <hyperlink ref="C5" r:id="rId5" xr:uid="{80FBAC2B-CD83-4D3B-8BCB-0BFF059C9B09}"/>
+    <hyperlink ref="C6" r:id="rId6" xr:uid="{A472254A-DB72-4F80-8E3F-549AE130CAFE}"/>
+    <hyperlink ref="C11" r:id="rId7" xr:uid="{3A26B573-E34D-469A-A519-C54C4E3D42C0}"/>
+    <hyperlink ref="C12" r:id="rId8" xr:uid="{669AE46F-78EB-41F5-A3DF-EAD27728EBA6}"/>
+    <hyperlink ref="C13" r:id="rId9" xr:uid="{4E218C59-F2C4-4892-A27C-5AFA85EDCA52}"/>
+    <hyperlink ref="C9" r:id="rId10" xr:uid="{733216EA-AAEC-4C8C-B3A9-ADA8A4D0B204}"/>
+    <hyperlink ref="C7" r:id="rId11" xr:uid="{AF2110D2-291F-442A-A5E5-57541CFF8277}"/>
+    <hyperlink ref="C8" r:id="rId12" xr:uid="{7A253563-3D9D-46CC-BC1C-DDD198212179}"/>
   </hyperlinks>
   <pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
-  <legacyDrawing r:id="rId2"/>
+  <legacyDrawing r:id="rId13"/>
 </worksheet>
 </file>
</xml_diff>